<commit_message>
First round of critique
Automated migration updates generated by Experience Modernization Agent.

Changed files (10):
- blocks/section-metadata/section-metadata.css
- blocks/section-metadata/section-metadata.js
- styles/brand.css
- styles/fonts.css
- styles/styles.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/reports/en.report.json
- tools/importer/reports/import-homepage.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>en.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","hero-banner","cards-nav","columns-media","columns-media","cards-feature","cards-news","cards-event","cards-stats","carousel-stories"]</t>
+    <t>["hero-banner","hero-banner","cards-nav","columns-media","columns-media","columns-media","columns-media","cards-feature","cards-news","cards-event","cards-stats","carousel-stories"]</t>
   </si>
   <si>
     <t>en</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-08-06T17:48:45.299Z</t>
+    <t>2026-08-06T18:44:40.253Z</t>
   </si>
   <si>
     <t>Atlas Copco Group Homepage</t>

</xml_diff>